<commit_message>
results for storage opt-all
</commit_message>
<xml_diff>
--- a/pidsg25Evaluation.xlsx
+++ b/pidsg25Evaluation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/debdeeppaul/Documents/Procurement/PIDSG25/pricesaa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79A63B66-53D6-D043-A3B5-DBDB77D7CC94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0D216AC-73DF-0546-A26B-53EE8CBABBD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15680" tabRatio="500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15680" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="from_alvin" sheetId="1" r:id="rId1"/>
@@ -485,17 +485,17 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -15907,10 +15907,10 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="21"/>
+      <c r="C3" s="23"/>
       <c r="D3" s="1">
         <v>45383</v>
       </c>
@@ -16372,10 +16372,10 @@
       </c>
     </row>
     <row r="14" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="21"/>
+      <c r="C14" s="23"/>
       <c r="D14" s="1">
         <v>45748</v>
       </c>
@@ -19518,7 +19518,7 @@
       </c>
     </row>
     <row r="2" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="H2" s="22" t="s">
+      <c r="H2" s="24" t="s">
         <v>58</v>
       </c>
       <c r="I2">
@@ -19529,7 +19529,7 @@
       </c>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="H3" s="22"/>
+      <c r="H3" s="24"/>
       <c r="I3">
         <v>2116045</v>
       </c>
@@ -21757,7 +21757,7 @@
       </c>
     </row>
     <row r="2" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="H2" s="22" t="s">
+      <c r="H2" s="24" t="s">
         <v>58</v>
       </c>
       <c r="I2">
@@ -21768,7 +21768,7 @@
       </c>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="H3" s="22"/>
+      <c r="H3" s="24"/>
       <c r="I3">
         <v>2116045</v>
       </c>
@@ -26599,7 +26599,7 @@
       </c>
     </row>
     <row r="130" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="I130" s="22" t="s">
+      <c r="I130" s="24" t="s">
         <v>58</v>
       </c>
       <c r="J130">
@@ -26610,7 +26610,7 @@
       </c>
     </row>
     <row r="131" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="I131" s="22"/>
+      <c r="I131" s="24"/>
       <c r="J131">
         <v>2116045</v>
       </c>
@@ -30756,11 +30756,11 @@
         <f t="shared" si="14"/>
         <v>-550.00000005873244</v>
       </c>
-      <c r="P49" s="24" t="s">
+      <c r="P49" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="Q49" s="23"/>
-      <c r="R49" s="23"/>
+      <c r="Q49" s="21"/>
+      <c r="R49" s="21"/>
     </row>
     <row r="50" spans="1:19" ht="16" x14ac:dyDescent="0.2">
       <c r="B50" s="17">
@@ -30800,11 +30800,11 @@
         <f t="shared" si="14"/>
         <v>-550.00000008036147</v>
       </c>
-      <c r="P50" s="24" t="s">
+      <c r="P50" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="Q50" s="23"/>
-      <c r="R50" s="23"/>
+      <c r="Q50" s="21"/>
+      <c r="R50" s="21"/>
     </row>
     <row r="51" spans="1:19" x14ac:dyDescent="0.2">
       <c r="K51" t="s">
@@ -30818,49 +30818,49 @@
         <f>SUM(M39:M50)</f>
         <v>-6271.3727227715071</v>
       </c>
-      <c r="P51" s="23">
+      <c r="P51" s="21">
         <v>2768</v>
       </c>
-      <c r="Q51" s="23">
+      <c r="Q51" s="21">
         <f>P51*(1-R47/100)</f>
         <v>2653.0912938133069</v>
       </c>
-      <c r="R51" s="23">
+      <c r="R51" s="21">
         <f>P51-Q51</f>
         <v>114.90870618669305</v>
       </c>
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="P52" s="23">
+      <c r="P52" s="21">
         <v>30.7</v>
       </c>
-      <c r="Q52" s="23">
+      <c r="Q52" s="21">
         <f>P52*(1-R41/100)</f>
         <v>12.319956606941059</v>
       </c>
-      <c r="R52" s="23">
+      <c r="R52" s="21">
         <f>P52-Q52</f>
         <v>18.380043393058941</v>
       </c>
     </row>
     <row r="53" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="P53" s="23">
+      <c r="P53" s="21">
         <f>SUM(P51:P52)</f>
         <v>2798.7</v>
       </c>
-      <c r="Q53" s="23">
+      <c r="Q53" s="21">
         <f>SUM(Q51:Q52)</f>
         <v>2665.4112504202481</v>
       </c>
-      <c r="R53" s="23">
+      <c r="R53" s="21">
         <f>SUM(R51:R52)</f>
         <v>133.28874957975199</v>
       </c>
     </row>
     <row r="54" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="P54" s="23"/>
-      <c r="Q54" s="23"/>
-      <c r="R54" s="23"/>
+      <c r="P54" s="21"/>
+      <c r="Q54" s="21"/>
+      <c r="R54" s="21"/>
     </row>
     <row r="56" spans="1:19" x14ac:dyDescent="0.2">
       <c r="B56" s="9" t="s">
@@ -31634,7 +31634,7 @@
       </c>
     </row>
     <row r="130" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="I130" s="22" t="s">
+      <c r="I130" s="24" t="s">
         <v>58</v>
       </c>
       <c r="J130">
@@ -31645,7 +31645,7 @@
       </c>
     </row>
     <row r="131" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="I131" s="22"/>
+      <c r="I131" s="24"/>
       <c r="J131">
         <v>2116045</v>
       </c>

</xml_diff>